<commit_message>
Update Notebook, README.md & result files
</commit_message>
<xml_diff>
--- a/results/submission_predictions.xlsx
+++ b/results/submission_predictions.xlsx
@@ -16,10 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -49,9 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1571,7 +1567,7 @@
         <v>0.03553853556513786</v>
       </c>
       <c r="F2" t="n">
-        <v>0.03609273582696915</v>
+        <v>0.03609274327754974</v>
       </c>
       <c r="G2" t="n">
         <v>0.03546727076172829</v>
@@ -1583,7 +1579,7 @@
         <v>0.03462072461843491</v>
       </c>
       <c r="J2" t="n">
-        <v>0.03485633060336113</v>
+        <v>0.03485633432865143</v>
       </c>
       <c r="K2" t="n">
         <v>0.03422610834240913</v>
@@ -1685,13 +1681,13 @@
         <v>0.08294537663459778</v>
       </c>
       <c r="AR2" t="n">
-        <v>0.1072399839758873</v>
+        <v>0.1072399914264679</v>
       </c>
       <c r="AS2" t="n">
         <v>0.1139924004673958</v>
       </c>
       <c r="AT2" t="n">
-        <v>0.114914558827877</v>
+        <v>0.1149145662784576</v>
       </c>
       <c r="AU2" t="n">
         <v>0.1169358789920807</v>
@@ -1727,7 +1723,7 @@
         <v>0.1017294079065323</v>
       </c>
       <c r="BF2" t="n">
-        <v>0.1351375430822372</v>
+        <v>0.1351375579833984</v>
       </c>
       <c r="BG2" t="n">
         <v>0.1371277421712875</v>
@@ -1742,7 +1738,7 @@
         <v>0.1337656676769257</v>
       </c>
       <c r="BK2" t="n">
-        <v>0.1279070228338242</v>
+        <v>0.1279070377349854</v>
       </c>
       <c r="BL2" t="n">
         <v>0.1275920271873474</v>
@@ -1757,7 +1753,7 @@
         <v>0.1247401759028435</v>
       </c>
       <c r="BP2" t="n">
-        <v>0.1169500574469566</v>
+        <v>0.1169500648975372</v>
       </c>
       <c r="BQ2" t="n">
         <v>0.1164049580693245</v>
@@ -1883,7 +1879,7 @@
         <v>0.1948543637990952</v>
       </c>
       <c r="DF2" t="n">
-        <v>0.1894200891256332</v>
+        <v>0.1894201040267944</v>
       </c>
       <c r="DG2" t="n">
         <v>0.1865202188491821</v>
@@ -1898,7 +1894,7 @@
         <v>0.2457068562507629</v>
       </c>
       <c r="DK2" t="n">
-        <v>0.2429618239402771</v>
+        <v>0.2429618388414383</v>
       </c>
       <c r="DL2" t="n">
         <v>0.2353169769048691</v>
@@ -2012,7 +2008,7 @@
         <v>0.246431291103363</v>
       </c>
       <c r="EW2" t="n">
-        <v>0.2465380728244781</v>
+        <v>0.2465380877256393</v>
       </c>
       <c r="EX2" t="n">
         <v>0.2465481609106064</v>
@@ -2066,7 +2062,7 @@
         <v>0.2864341139793396</v>
       </c>
       <c r="FO2" t="n">
-        <v>0.2868529558181763</v>
+        <v>0.2868529856204987</v>
       </c>
       <c r="FP2" t="n">
         <v>0.2789511382579803</v>
@@ -2117,7 +2113,7 @@
         <v>0.3034860193729401</v>
       </c>
       <c r="GF2" t="n">
-        <v>0.3017010390758514</v>
+        <v>0.3017010688781738</v>
       </c>
       <c r="GG2" t="n">
         <v>0.3001542687416077</v>
@@ -2156,7 +2152,7 @@
         <v>0.3265229165554047</v>
       </c>
       <c r="GS2" t="n">
-        <v>0.3249167203903198</v>
+        <v>0.3249167501926422</v>
       </c>
       <c r="GT2" t="n">
         <v>0.3261618912220001</v>
@@ -2183,7 +2179,7 @@
         <v>0.3482560217380524</v>
       </c>
       <c r="HB2" t="n">
-        <v>0.3604863584041595</v>
+        <v>0.3604863882064819</v>
       </c>
       <c r="HC2" t="n">
         <v>0.3553192019462585</v>
@@ -2230,8 +2226,10 @@
       <c r="HQ2" t="n">
         <v>0.3446680307388306</v>
       </c>
-      <c r="HR2" s="1" t="n">
-        <v>55512</v>
+      <c r="HR2" t="inlineStr">
+        <is>
+          <t>24/12/2051</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -2241,7 +2239,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.02405373938381672</v>
+        <v>0.02405374124646187</v>
       </c>
       <c r="C3" t="n">
         <v>0.03270313516259193</v>
@@ -2286,19 +2284,19 @@
         <v>0.04883988574147224</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.06013626605272293</v>
+        <v>0.06013627350330353</v>
       </c>
       <c r="R3" t="n">
         <v>0.06284879893064499</v>
       </c>
       <c r="S3" t="n">
-        <v>0.06389123946428299</v>
+        <v>0.06389124691486359</v>
       </c>
       <c r="T3" t="n">
-        <v>0.06511685997247696</v>
+        <v>0.06511686742305756</v>
       </c>
       <c r="U3" t="n">
-        <v>0.06285393238067627</v>
+        <v>0.06285393983125687</v>
       </c>
       <c r="V3" t="n">
         <v>0.06368936598300934</v>
@@ -2322,10 +2320,10 @@
         <v>0.05685501918196678</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.05827780067920685</v>
+        <v>0.05827780440449715</v>
       </c>
       <c r="AD3" t="n">
-        <v>0.08020353317260742</v>
+        <v>0.08020354062318802</v>
       </c>
       <c r="AE3" t="n">
         <v>0.09205266088247299</v>
@@ -2367,7 +2365,7 @@
         <v>0.08378931879997253</v>
       </c>
       <c r="AR3" t="n">
-        <v>0.1091591417789459</v>
+        <v>0.1091591492295265</v>
       </c>
       <c r="AS3" t="n">
         <v>0.1161635741591454</v>
@@ -2385,7 +2383,7 @@
         <v>0.1125217750668526</v>
       </c>
       <c r="AX3" t="n">
-        <v>0.1130005866289139</v>
+        <v>0.1130005940794945</v>
       </c>
       <c r="AY3" t="n">
         <v>0.1121794953942299</v>
@@ -2400,7 +2398,7 @@
         <v>0.1026151031255722</v>
       </c>
       <c r="BC3" t="n">
-        <v>0.1009214073419571</v>
+        <v>0.1009214147925377</v>
       </c>
       <c r="BD3" t="n">
         <v>0.09962698817253113</v>
@@ -2436,7 +2434,7 @@
         <v>0.1247759908437729</v>
       </c>
       <c r="BO3" t="n">
-        <v>0.1260892152786255</v>
+        <v>0.1260892301797867</v>
       </c>
       <c r="BP3" t="n">
         <v>0.1180642545223236</v>
@@ -2460,7 +2458,7 @@
         <v>0.1656215339899063</v>
       </c>
       <c r="BW3" t="n">
-        <v>0.1656820327043533</v>
+        <v>0.1656820476055145</v>
       </c>
       <c r="BX3" t="n">
         <v>0.1639607101678848</v>
@@ -2502,7 +2500,7 @@
         <v>0.1925187855958939</v>
       </c>
       <c r="CK3" t="n">
-        <v>0.1886909157037735</v>
+        <v>0.1886909306049347</v>
       </c>
       <c r="CL3" t="n">
         <v>0.1850903928279877</v>
@@ -2577,16 +2575,16 @@
         <v>0.189191535115242</v>
       </c>
       <c r="DJ3" t="n">
-        <v>0.2488144785165787</v>
+        <v>0.2488144934177399</v>
       </c>
       <c r="DK3" t="n">
         <v>0.2457433938980103</v>
       </c>
       <c r="DL3" t="n">
-        <v>0.2378329932689667</v>
+        <v>0.2378330081701279</v>
       </c>
       <c r="DM3" t="n">
-        <v>0.2362802028656006</v>
+        <v>0.2362802177667618</v>
       </c>
       <c r="DN3" t="n">
         <v>0.2294298559427261</v>
@@ -2601,7 +2599,7 @@
         <v>0.2190182507038116</v>
       </c>
       <c r="DR3" t="n">
-        <v>0.2176065593957901</v>
+        <v>0.2176065891981125</v>
       </c>
       <c r="DS3" t="n">
         <v>0.2147616446018219</v>
@@ -2631,7 +2629,7 @@
         <v>0.2474002242088318</v>
       </c>
       <c r="EB3" t="n">
-        <v>0.2468252182006836</v>
+        <v>0.2468252331018448</v>
       </c>
       <c r="EC3" t="n">
         <v>0.241018608212471</v>
@@ -2706,7 +2704,7 @@
         <v>0.2834609150886536</v>
       </c>
       <c r="FA3" t="n">
-        <v>0.2839841544628143</v>
+        <v>0.2839841842651367</v>
       </c>
       <c r="FB3" t="n">
         <v>0.2734586000442505</v>
@@ -2748,7 +2746,7 @@
         <v>0.2875897884368896</v>
       </c>
       <c r="FO3" t="n">
-        <v>0.2879283130168915</v>
+        <v>0.2879283428192139</v>
       </c>
       <c r="FP3" t="n">
         <v>0.2799690961837769</v>
@@ -2910,10 +2908,12 @@
         <v>0.3569716811180115</v>
       </c>
       <c r="HQ3" t="n">
-        <v>0.3456933796405792</v>
-      </c>
-      <c r="HR3" s="1" t="n">
-        <v>55513</v>
+        <v>0.3456934094429016</v>
+      </c>
+      <c r="HR3" t="inlineStr">
+        <is>
+          <t>26/12/2051</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -2923,40 +2923,40 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.02440594509243965</v>
+        <v>0.02440594881772995</v>
       </c>
       <c r="C4" t="n">
-        <v>0.03310086950659752</v>
+        <v>0.03310087323188782</v>
       </c>
       <c r="D4" t="n">
-        <v>0.03520696237683296</v>
+        <v>0.03520696610212326</v>
       </c>
       <c r="E4" t="n">
-        <v>0.03676065802574158</v>
+        <v>0.03676066175103188</v>
       </c>
       <c r="F4" t="n">
-        <v>0.03725502267479897</v>
+        <v>0.03725502640008926</v>
       </c>
       <c r="G4" t="n">
         <v>0.03656097874045372</v>
       </c>
       <c r="H4" t="n">
-        <v>0.03599255904555321</v>
+        <v>0.03599256277084351</v>
       </c>
       <c r="I4" t="n">
         <v>0.03564152866601944</v>
       </c>
       <c r="J4" t="n">
-        <v>0.03585303574800491</v>
+        <v>0.03585303947329521</v>
       </c>
       <c r="K4" t="n">
-        <v>0.03517654538154602</v>
+        <v>0.03517654910683632</v>
       </c>
       <c r="L4" t="n">
         <v>0.03415499627590179</v>
       </c>
       <c r="M4" t="n">
-        <v>0.03315304592251778</v>
+        <v>0.03315304964780807</v>
       </c>
       <c r="N4" t="n">
         <v>0.03307050094008446</v>
@@ -2965,46 +2965,46 @@
         <v>0.03364849463105202</v>
       </c>
       <c r="P4" t="n">
-        <v>0.0494098886847496</v>
+        <v>0.0494098924100399</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.0607617199420929</v>
+        <v>0.06076172739267349</v>
       </c>
       <c r="R4" t="n">
-        <v>0.06350771337747574</v>
+        <v>0.06350772082805634</v>
       </c>
       <c r="S4" t="n">
         <v>0.0645090639591217</v>
       </c>
       <c r="T4" t="n">
-        <v>0.0657382607460022</v>
+        <v>0.06573826819658279</v>
       </c>
       <c r="U4" t="n">
-        <v>0.06342463940382004</v>
+        <v>0.06342464685440063</v>
       </c>
       <c r="V4" t="n">
-        <v>0.0642491951584816</v>
+        <v>0.06424920260906219</v>
       </c>
       <c r="W4" t="n">
-        <v>0.06379463523626328</v>
+        <v>0.06379464268684387</v>
       </c>
       <c r="X4" t="n">
         <v>0.06324773281812668</v>
       </c>
       <c r="Y4" t="n">
-        <v>0.06282945722341537</v>
+        <v>0.06282946467399597</v>
       </c>
       <c r="Z4" t="n">
-        <v>0.0597500167787075</v>
+        <v>0.0597500242292881</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.05747367441654205</v>
+        <v>0.05747367814183235</v>
       </c>
       <c r="AB4" t="n">
         <v>0.05729715153574944</v>
       </c>
       <c r="AC4" t="n">
-        <v>0.05871054530143738</v>
+        <v>0.05871054902672768</v>
       </c>
       <c r="AD4" t="n">
         <v>0.08093959093093872</v>
@@ -3013,61 +3013,61 @@
         <v>0.09287602454423904</v>
       </c>
       <c r="AF4" t="n">
-        <v>0.09291137009859085</v>
+        <v>0.09291137754917145</v>
       </c>
       <c r="AG4" t="n">
-        <v>0.09494400024414062</v>
+        <v>0.09494400769472122</v>
       </c>
       <c r="AH4" t="n">
-        <v>0.09517054259777069</v>
+        <v>0.09517055004835129</v>
       </c>
       <c r="AI4" t="n">
-        <v>0.09449223428964615</v>
+        <v>0.09449224919080734</v>
       </c>
       <c r="AJ4" t="n">
-        <v>0.09135963767766953</v>
+        <v>0.09135964512825012</v>
       </c>
       <c r="AK4" t="n">
         <v>0.09038989990949631</v>
       </c>
       <c r="AL4" t="n">
-        <v>0.09065088629722595</v>
+        <v>0.09065089374780655</v>
       </c>
       <c r="AM4" t="n">
         <v>0.0876496210694313</v>
       </c>
       <c r="AN4" t="n">
-        <v>0.08344297111034393</v>
+        <v>0.08344297856092453</v>
       </c>
       <c r="AO4" t="n">
-        <v>0.08146142959594727</v>
+        <v>0.08146143704652786</v>
       </c>
       <c r="AP4" t="n">
         <v>0.08362265676259995</v>
       </c>
       <c r="AQ4" t="n">
-        <v>0.08433092385530472</v>
+        <v>0.08433093130588531</v>
       </c>
       <c r="AR4" t="n">
         <v>0.1100423559546471</v>
       </c>
       <c r="AS4" t="n">
-        <v>0.1171707063913345</v>
+        <v>0.1171707138419151</v>
       </c>
       <c r="AT4" t="n">
-        <v>0.1179169267416</v>
+        <v>0.1179169341921806</v>
       </c>
       <c r="AU4" t="n">
         <v>0.1195550784468651</v>
       </c>
       <c r="AV4" t="n">
-        <v>0.1175246983766556</v>
+        <v>0.1175247058272362</v>
       </c>
       <c r="AW4" t="n">
-        <v>0.1133393347263336</v>
+        <v>0.1133393421769142</v>
       </c>
       <c r="AX4" t="n">
-        <v>0.1138123497366905</v>
+        <v>0.1138123646378517</v>
       </c>
       <c r="AY4" t="n">
         <v>0.1129530891776085</v>
@@ -3076,37 +3076,37 @@
         <v>0.1115578413009644</v>
       </c>
       <c r="BA4" t="n">
-        <v>0.1078924834728241</v>
+        <v>0.1078924909234047</v>
       </c>
       <c r="BB4" t="n">
-        <v>0.1032412052154541</v>
+        <v>0.1032412126660347</v>
       </c>
       <c r="BC4" t="n">
         <v>0.1015353351831436</v>
       </c>
       <c r="BD4" t="n">
-        <v>0.1002434492111206</v>
+        <v>0.1002434566617012</v>
       </c>
       <c r="BE4" t="n">
-        <v>0.1032748520374298</v>
+        <v>0.1032748594880104</v>
       </c>
       <c r="BF4" t="n">
         <v>0.1383955925703049</v>
       </c>
       <c r="BG4" t="n">
-        <v>0.140576496720314</v>
+        <v>0.1405765116214752</v>
       </c>
       <c r="BH4" t="n">
-        <v>0.1400087475776672</v>
+        <v>0.1400087624788284</v>
       </c>
       <c r="BI4" t="n">
-        <v>0.1366239041090012</v>
+        <v>0.1366239190101624</v>
       </c>
       <c r="BJ4" t="n">
-        <v>0.1367008835077286</v>
+        <v>0.1367008984088898</v>
       </c>
       <c r="BK4" t="n">
-        <v>0.1305189579725266</v>
+        <v>0.1305189728736877</v>
       </c>
       <c r="BL4" t="n">
         <v>0.1299921125173569</v>
@@ -3118,37 +3118,37 @@
         <v>0.1255935877561569</v>
       </c>
       <c r="BO4" t="n">
-        <v>0.1268680542707443</v>
+        <v>0.1268680691719055</v>
       </c>
       <c r="BP4" t="n">
-        <v>0.1187395453453064</v>
+        <v>0.118739552795887</v>
       </c>
       <c r="BQ4" t="n">
-        <v>0.1180970594286919</v>
+        <v>0.1180970668792725</v>
       </c>
       <c r="BR4" t="n">
-        <v>0.1174595803022385</v>
+        <v>0.1174595877528191</v>
       </c>
       <c r="BS4" t="n">
-        <v>0.1173398569226265</v>
+        <v>0.1173398643732071</v>
       </c>
       <c r="BT4" t="n">
-        <v>0.1730543375015259</v>
+        <v>0.1730543524026871</v>
       </c>
       <c r="BU4" t="n">
-        <v>0.1711735725402832</v>
+        <v>0.1711735874414444</v>
       </c>
       <c r="BV4" t="n">
-        <v>0.1670238077640533</v>
+        <v>0.1670238226652145</v>
       </c>
       <c r="BW4" t="n">
-        <v>0.166950985789299</v>
+        <v>0.1669510155916214</v>
       </c>
       <c r="BX4" t="n">
         <v>0.1651178598403931</v>
       </c>
       <c r="BY4" t="n">
-        <v>0.1610991060733795</v>
+        <v>0.1610991209745407</v>
       </c>
       <c r="BZ4" t="n">
         <v>0.157201960682869</v>
@@ -3160,34 +3160,34 @@
         <v>0.1523000150918961</v>
       </c>
       <c r="CC4" t="n">
-        <v>0.1481921076774597</v>
+        <v>0.1481921225786209</v>
       </c>
       <c r="CD4" t="n">
-        <v>0.1445032060146332</v>
+        <v>0.1445032209157944</v>
       </c>
       <c r="CE4" t="n">
-        <v>0.1378577202558517</v>
+        <v>0.1378577351570129</v>
       </c>
       <c r="CF4" t="n">
-        <v>0.137981042265892</v>
+        <v>0.1379810571670532</v>
       </c>
       <c r="CG4" t="n">
-        <v>0.1412186473608017</v>
+        <v>0.1412186622619629</v>
       </c>
       <c r="CH4" t="n">
-        <v>0.1989464610815048</v>
+        <v>0.198946475982666</v>
       </c>
       <c r="CI4" t="n">
-        <v>0.1968491971492767</v>
+        <v>0.1968492120504379</v>
       </c>
       <c r="CJ4" t="n">
-        <v>0.1940256357192993</v>
+        <v>0.1940256506204605</v>
       </c>
       <c r="CK4" t="n">
-        <v>0.1900310665369034</v>
+        <v>0.1900310814380646</v>
       </c>
       <c r="CL4" t="n">
-        <v>0.1863956451416016</v>
+        <v>0.1863956600427628</v>
       </c>
       <c r="CM4" t="n">
         <v>0.1797317117452621</v>
@@ -3205,28 +3205,28 @@
         <v>0.1732037663459778</v>
       </c>
       <c r="CR4" t="n">
-        <v>0.1604510545730591</v>
+        <v>0.1604510694742203</v>
       </c>
       <c r="CS4" t="n">
         <v>0.1579433530569077</v>
       </c>
       <c r="CT4" t="n">
-        <v>0.157959908246994</v>
+        <v>0.1579599231481552</v>
       </c>
       <c r="CU4" t="n">
-        <v>0.1641116142272949</v>
+        <v>0.1641116291284561</v>
       </c>
       <c r="CV4" t="n">
-        <v>0.234425276517868</v>
+        <v>0.2344253063201904</v>
       </c>
       <c r="CW4" t="n">
-        <v>0.2218238860368729</v>
+        <v>0.2218239009380341</v>
       </c>
       <c r="CX4" t="n">
         <v>0.2217310965061188</v>
       </c>
       <c r="CY4" t="n">
-        <v>0.2200888246297836</v>
+        <v>0.2200888395309448</v>
       </c>
       <c r="CZ4" t="n">
         <v>0.2108585834503174</v>
@@ -3238,7 +3238,7 @@
         <v>0.2078601270914078</v>
       </c>
       <c r="DC4" t="n">
-        <v>0.2033772766590118</v>
+        <v>0.203377291560173</v>
       </c>
       <c r="DD4" t="n">
         <v>0.2028948664665222</v>
@@ -3250,10 +3250,10 @@
         <v>0.1915483474731445</v>
       </c>
       <c r="DG4" t="n">
-        <v>0.1884981095790863</v>
+        <v>0.1884981393814087</v>
       </c>
       <c r="DH4" t="n">
-        <v>0.187359482049942</v>
+        <v>0.1873594969511032</v>
       </c>
       <c r="DI4" t="n">
         <v>0.1899510324001312</v>
@@ -3262,22 +3262,22 @@
         <v>0.2506311237812042</v>
       </c>
       <c r="DK4" t="n">
-        <v>0.2474002540111542</v>
+        <v>0.2474002838134766</v>
       </c>
       <c r="DL4" t="n">
-        <v>0.2393234223127365</v>
+        <v>0.2393234372138977</v>
       </c>
       <c r="DM4" t="n">
-        <v>0.2377154678106308</v>
+        <v>0.237715482711792</v>
       </c>
       <c r="DN4" t="n">
-        <v>0.2307732403278351</v>
+        <v>0.2307732552289963</v>
       </c>
       <c r="DO4" t="n">
-        <v>0.2318024784326553</v>
+        <v>0.2318024933338165</v>
       </c>
       <c r="DP4" t="n">
-        <v>0.2260192483663559</v>
+        <v>0.2260192632675171</v>
       </c>
       <c r="DQ4" t="n">
         <v>0.2200573980808258</v>
@@ -3286,7 +3286,7 @@
         <v>0.2185904085636139</v>
       </c>
       <c r="DS4" t="n">
-        <v>0.2156789898872375</v>
+        <v>0.2156790047883987</v>
       </c>
       <c r="DT4" t="n">
         <v>0.2110443115234375</v>
@@ -3301,28 +3301,28 @@
         <v>0.2140649408102036</v>
       </c>
       <c r="DX4" t="n">
-        <v>0.2673621773719788</v>
+        <v>0.2673622071743011</v>
       </c>
       <c r="DY4" t="n">
-        <v>0.2573992908000946</v>
+        <v>0.257399320602417</v>
       </c>
       <c r="DZ4" t="n">
         <v>0.255962610244751</v>
       </c>
       <c r="EA4" t="n">
-        <v>0.2486803233623505</v>
+        <v>0.2486803382635117</v>
       </c>
       <c r="EB4" t="n">
-        <v>0.2480099946260452</v>
+        <v>0.2480100095272064</v>
       </c>
       <c r="EC4" t="n">
-        <v>0.2421408146619797</v>
+        <v>0.2421408444643021</v>
       </c>
       <c r="ED4" t="n">
         <v>0.2394766062498093</v>
       </c>
       <c r="EE4" t="n">
-        <v>0.2380269467830658</v>
+        <v>0.2380269765853882</v>
       </c>
       <c r="EF4" t="n">
         <v>0.2357321232557297</v>
@@ -3346,13 +3346,13 @@
         <v>0.2775877118110657</v>
       </c>
       <c r="EM4" t="n">
-        <v>0.2743952870368958</v>
+        <v>0.2743953168392181</v>
       </c>
       <c r="EN4" t="n">
-        <v>0.2702313363552094</v>
+        <v>0.2702313661575317</v>
       </c>
       <c r="EO4" t="n">
-        <v>0.2634848654270172</v>
+        <v>0.2634848952293396</v>
       </c>
       <c r="EP4" t="n">
         <v>0.2666943967342377</v>
@@ -3376,7 +3376,7 @@
         <v>0.2481397092342377</v>
       </c>
       <c r="EW4" t="n">
-        <v>0.248043566942215</v>
+        <v>0.2480435818433762</v>
       </c>
       <c r="EX4" t="n">
         <v>0.2479010969400406</v>
@@ -3394,7 +3394,7 @@
         <v>0.2742069363594055</v>
       </c>
       <c r="FC4" t="n">
-        <v>0.2765864729881287</v>
+        <v>0.276586502790451</v>
       </c>
       <c r="FD4" t="n">
         <v>0.2670504450798035</v>
@@ -3418,16 +3418,16 @@
         <v>0.2614202797412872</v>
       </c>
       <c r="FK4" t="n">
-        <v>0.2634250223636627</v>
+        <v>0.2634250521659851</v>
       </c>
       <c r="FL4" t="n">
-        <v>0.2731781601905823</v>
+        <v>0.2731781899929047</v>
       </c>
       <c r="FM4" t="n">
         <v>0.28343465924263</v>
       </c>
       <c r="FN4" t="n">
-        <v>0.2884003818035126</v>
+        <v>0.288400411605835</v>
       </c>
       <c r="FO4" t="n">
         <v>0.2886927425861359</v>
@@ -3451,10 +3451,10 @@
         <v>0.2800556123256683</v>
       </c>
       <c r="FV4" t="n">
-        <v>0.2818794846534729</v>
+        <v>0.2818795144557953</v>
       </c>
       <c r="FW4" t="n">
-        <v>0.2822479009628296</v>
+        <v>0.282247930765152</v>
       </c>
       <c r="FX4" t="n">
         <v>0.2814530730247498</v>
@@ -3469,7 +3469,7 @@
         <v>0.3110823929309845</v>
       </c>
       <c r="GB4" t="n">
-        <v>0.3043985664844513</v>
+        <v>0.3043985962867737</v>
       </c>
       <c r="GC4" t="n">
         <v>0.3050969541072845</v>
@@ -3487,10 +3487,10 @@
         <v>0.302635669708252</v>
       </c>
       <c r="GH4" t="n">
-        <v>0.2989324629306793</v>
+        <v>0.2989324927330017</v>
       </c>
       <c r="GI4" t="n">
-        <v>0.2996359467506409</v>
+        <v>0.2996359765529633</v>
       </c>
       <c r="GJ4" t="n">
         <v>0.2999996840953827</v>
@@ -3502,16 +3502,16 @@
         <v>0.3104371726512909</v>
       </c>
       <c r="GM4" t="n">
-        <v>0.3168556988239288</v>
+        <v>0.3168557286262512</v>
       </c>
       <c r="GN4" t="n">
         <v>0.3321373164653778</v>
       </c>
       <c r="GO4" t="n">
-        <v>0.3398800790309906</v>
+        <v>0.339880108833313</v>
       </c>
       <c r="GP4" t="n">
-        <v>0.3328006863594055</v>
+        <v>0.3328007161617279</v>
       </c>
       <c r="GQ4" t="n">
         <v>0.3298621475696564</v>
@@ -3535,10 +3535,10 @@
         <v>0.3230894505977631</v>
       </c>
       <c r="GX4" t="n">
-        <v>0.3241716623306274</v>
+        <v>0.3241716921329498</v>
       </c>
       <c r="GY4" t="n">
-        <v>0.3244462013244629</v>
+        <v>0.3244462311267853</v>
       </c>
       <c r="GZ4" t="n">
         <v>0.3376578986644745</v>
@@ -3553,13 +3553,13 @@
         <v>0.3573117852210999</v>
       </c>
       <c r="HD4" t="n">
-        <v>0.3454219698905945</v>
+        <v>0.3454219996929169</v>
       </c>
       <c r="HE4" t="n">
         <v>0.3406133651733398</v>
       </c>
       <c r="HF4" t="n">
-        <v>0.3421693444252014</v>
+        <v>0.3421693742275238</v>
       </c>
       <c r="HG4" t="n">
         <v>0.3487009406089783</v>
@@ -3571,13 +3571,13 @@
         <v>0.3458665907382965</v>
       </c>
       <c r="HJ4" t="n">
-        <v>0.3484143614768982</v>
+        <v>0.3484143912792206</v>
       </c>
       <c r="HK4" t="n">
-        <v>0.3421349227428436</v>
+        <v>0.342134952545166</v>
       </c>
       <c r="HL4" t="n">
-        <v>0.3438485264778137</v>
+        <v>0.3438485562801361</v>
       </c>
       <c r="HM4" t="n">
         <v>0.3408194780349731</v>
@@ -3589,13 +3589,15 @@
         <v>0.3782960772514343</v>
       </c>
       <c r="HP4" t="n">
-        <v>0.3580786883831024</v>
+        <v>0.3580787181854248</v>
       </c>
       <c r="HQ4" t="n">
         <v>0.3464901149272919</v>
       </c>
-      <c r="HR4" s="1" t="n">
-        <v>55514</v>
+      <c r="HR4" t="inlineStr">
+        <is>
+          <t>27/12/2051</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -3605,22 +3607,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02477490529417992</v>
+        <v>0.02477490715682507</v>
       </c>
       <c r="C5" t="n">
-        <v>0.03348959609866142</v>
+        <v>0.03348959982395172</v>
       </c>
       <c r="D5" t="n">
-        <v>0.03558918461203575</v>
+        <v>0.03558918833732605</v>
       </c>
       <c r="E5" t="n">
-        <v>0.03713205829262733</v>
+        <v>0.03713206201791763</v>
       </c>
       <c r="F5" t="n">
         <v>0.03760436549782753</v>
       </c>
       <c r="G5" t="n">
-        <v>0.03689340129494667</v>
+        <v>0.03689340502023697</v>
       </c>
       <c r="H5" t="n">
         <v>0.03631202504038811</v>
@@ -3629,46 +3631,46 @@
         <v>0.03596088662743568</v>
       </c>
       <c r="J5" t="n">
-        <v>0.03616899996995926</v>
+        <v>0.03616900369524956</v>
       </c>
       <c r="K5" t="n">
-        <v>0.03548309206962585</v>
+        <v>0.03548309579491615</v>
       </c>
       <c r="L5" t="n">
-        <v>0.03444059938192368</v>
+        <v>0.03444060310721397</v>
       </c>
       <c r="M5" t="n">
-        <v>0.03341441601514816</v>
+        <v>0.03341441974043846</v>
       </c>
       <c r="N5" t="n">
-        <v>0.03333155065774918</v>
+        <v>0.03333155438303947</v>
       </c>
       <c r="O5" t="n">
-        <v>0.03390952199697495</v>
+        <v>0.03390952572226524</v>
       </c>
       <c r="P5" t="n">
-        <v>0.04998867586255074</v>
+        <v>0.04998867958784103</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.06135455518960953</v>
+        <v>0.06135455891489983</v>
       </c>
       <c r="R5" t="n">
         <v>0.0641135647892952</v>
       </c>
       <c r="S5" t="n">
-        <v>0.065064437687397</v>
+        <v>0.0650644451379776</v>
       </c>
       <c r="T5" t="n">
-        <v>0.06629300862550735</v>
+        <v>0.06629301607608795</v>
       </c>
       <c r="U5" t="n">
-        <v>0.06393595784902573</v>
+        <v>0.06393596529960632</v>
       </c>
       <c r="V5" t="n">
         <v>0.06474974751472473</v>
       </c>
       <c r="W5" t="n">
-        <v>0.06427901983261108</v>
+        <v>0.06427902728319168</v>
       </c>
       <c r="X5" t="n">
         <v>0.06373234838247299</v>
@@ -3680,7 +3682,7 @@
         <v>0.06017992272973061</v>
       </c>
       <c r="AA5" t="n">
-        <v>0.05788280814886093</v>
+        <v>0.05788281187415123</v>
       </c>
       <c r="AB5" t="n">
         <v>0.05771336704492569</v>
@@ -3689,16 +3691,16 @@
         <v>0.05912180244922638</v>
       </c>
       <c r="AD5" t="n">
-        <v>0.08165702968835831</v>
+        <v>0.0816570371389389</v>
       </c>
       <c r="AE5" t="n">
         <v>0.09361825883388519</v>
       </c>
       <c r="AF5" t="n">
-        <v>0.09366682171821594</v>
+        <v>0.09366682916879654</v>
       </c>
       <c r="AG5" t="n">
-        <v>0.09562629461288452</v>
+        <v>0.09562630206346512</v>
       </c>
       <c r="AH5" t="n">
         <v>0.09585040062665939</v>
@@ -3707,13 +3709,13 @@
         <v>0.09515044838190079</v>
       </c>
       <c r="AJ5" t="n">
-        <v>0.09197987616062164</v>
+        <v>0.09197988361120224</v>
       </c>
       <c r="AK5" t="n">
         <v>0.09098777920007706</v>
       </c>
       <c r="AL5" t="n">
-        <v>0.09125534445047379</v>
+        <v>0.09125535190105438</v>
       </c>
       <c r="AM5" t="n">
         <v>0.08822953701019287</v>
@@ -3725,7 +3727,7 @@
         <v>0.08196645230054855</v>
       </c>
       <c r="AP5" t="n">
-        <v>0.08415248245000839</v>
+        <v>0.08415248990058899</v>
       </c>
       <c r="AQ5" t="n">
         <v>0.08484955877065659</v>
@@ -3734,28 +3736,28 @@
         <v>0.1108589917421341</v>
       </c>
       <c r="AS5" t="n">
-        <v>0.1180406883358955</v>
+        <v>0.1180407032370567</v>
       </c>
       <c r="AT5" t="n">
-        <v>0.1187440752983093</v>
+        <v>0.1187440901994705</v>
       </c>
       <c r="AU5" t="n">
-        <v>0.1202830150723457</v>
+        <v>0.1202830225229263</v>
       </c>
       <c r="AV5" t="n">
-        <v>0.1183508336544037</v>
+        <v>0.1183508411049843</v>
       </c>
       <c r="AW5" t="n">
         <v>0.1140555590391159</v>
       </c>
       <c r="AX5" t="n">
-        <v>0.1145311817526817</v>
+        <v>0.1145311892032623</v>
       </c>
       <c r="AY5" t="n">
-        <v>0.1136466041207314</v>
+        <v>0.113646611571312</v>
       </c>
       <c r="AZ5" t="n">
-        <v>0.1122476980090141</v>
+        <v>0.1122477054595947</v>
       </c>
       <c r="BA5" t="n">
         <v>0.1085412129759789</v>
@@ -3764,10 +3766,10 @@
         <v>0.1038171276450157</v>
       </c>
       <c r="BC5" t="n">
-        <v>0.1021154597401619</v>
+        <v>0.1021154671907425</v>
       </c>
       <c r="BD5" t="n">
-        <v>0.1008310168981552</v>
+        <v>0.1008310243487358</v>
       </c>
       <c r="BE5" t="n">
         <v>0.1038637906312943</v>
@@ -3776,13 +3778,13 @@
         <v>0.1392594128847122</v>
       </c>
       <c r="BG5" t="n">
-        <v>0.1415179520845413</v>
+        <v>0.1415179669857025</v>
       </c>
       <c r="BH5" t="n">
-        <v>0.1408963054418564</v>
+        <v>0.1408963203430176</v>
       </c>
       <c r="BI5" t="n">
-        <v>0.1374604552984238</v>
+        <v>0.137460470199585</v>
       </c>
       <c r="BJ5" t="n">
         <v>0.1375902742147446</v>
@@ -3803,10 +3805,10 @@
         <v>0.1275741904973984</v>
       </c>
       <c r="BP5" t="n">
-        <v>0.1193665042519569</v>
+        <v>0.1193665117025375</v>
       </c>
       <c r="BQ5" t="n">
-        <v>0.1187270283699036</v>
+        <v>0.1187270358204842</v>
       </c>
       <c r="BR5" t="n">
         <v>0.1180975437164307</v>
@@ -3815,10 +3817,10 @@
         <v>0.1179642900824547</v>
       </c>
       <c r="BT5" t="n">
-        <v>0.1742985844612122</v>
+        <v>0.1742985993623734</v>
       </c>
       <c r="BU5" t="n">
-        <v>0.1723891496658325</v>
+        <v>0.1723891645669937</v>
       </c>
       <c r="BV5" t="n">
         <v>0.1682400405406952</v>
@@ -3830,7 +3832,7 @@
         <v>0.1661363840103149</v>
       </c>
       <c r="BY5" t="n">
-        <v>0.1621057093143463</v>
+        <v>0.1621057242155075</v>
       </c>
       <c r="BZ5" t="n">
         <v>0.1581279933452606</v>
@@ -3857,28 +3859,28 @@
         <v>0.1419283300638199</v>
       </c>
       <c r="CH5" t="n">
-        <v>0.2002800852060318</v>
+        <v>0.200280100107193</v>
       </c>
       <c r="CI5" t="n">
-        <v>0.198260635137558</v>
+        <v>0.1982606649398804</v>
       </c>
       <c r="CJ5" t="n">
-        <v>0.1953572034835815</v>
+        <v>0.1953572183847427</v>
       </c>
       <c r="CK5" t="n">
-        <v>0.1912230551242828</v>
+        <v>0.191223070025444</v>
       </c>
       <c r="CL5" t="n">
         <v>0.1875691264867783</v>
       </c>
       <c r="CM5" t="n">
-        <v>0.180831715464592</v>
+        <v>0.1808317303657532</v>
       </c>
       <c r="CN5" t="n">
         <v>0.1813734620809555</v>
       </c>
       <c r="CO5" t="n">
-        <v>0.174965888261795</v>
+        <v>0.1749659031629562</v>
       </c>
       <c r="CP5" t="n">
         <v>0.1733799576759338</v>
@@ -3893,37 +3895,37 @@
         <v>0.1586896926164627</v>
       </c>
       <c r="CT5" t="n">
-        <v>0.1586892455816269</v>
+        <v>0.1586892604827881</v>
       </c>
       <c r="CU5" t="n">
         <v>0.1648840308189392</v>
       </c>
       <c r="CV5" t="n">
-        <v>0.2358627766370773</v>
+        <v>0.2358627915382385</v>
       </c>
       <c r="CW5" t="n">
-        <v>0.2233276814222336</v>
+        <v>0.2233276963233948</v>
       </c>
       <c r="CX5" t="n">
         <v>0.2230869382619858</v>
       </c>
       <c r="CY5" t="n">
-        <v>0.221435546875</v>
+        <v>0.2214355617761612</v>
       </c>
       <c r="CZ5" t="n">
         <v>0.2120961099863052</v>
       </c>
       <c r="DA5" t="n">
-        <v>0.2085774093866348</v>
+        <v>0.208577424287796</v>
       </c>
       <c r="DB5" t="n">
-        <v>0.208969920873642</v>
+        <v>0.2089699357748032</v>
       </c>
       <c r="DC5" t="n">
         <v>0.2043729573488235</v>
       </c>
       <c r="DD5" t="n">
-        <v>0.2038628160953522</v>
+        <v>0.2038628309965134</v>
       </c>
       <c r="DE5" t="n">
         <v>0.1982628107070923</v>
@@ -3938,13 +3940,13 @@
         <v>0.1881154328584671</v>
       </c>
       <c r="DI5" t="n">
-        <v>0.190725713968277</v>
+        <v>0.1907257437705994</v>
       </c>
       <c r="DJ5" t="n">
         <v>0.2522956728935242</v>
       </c>
       <c r="DK5" t="n">
-        <v>0.2489318996667862</v>
+        <v>0.2489319145679474</v>
       </c>
       <c r="DL5" t="n">
         <v>0.2407002151012421</v>
@@ -3956,7 +3958,7 @@
         <v>0.2320291697978973</v>
       </c>
       <c r="DO5" t="n">
-        <v>0.2329266220331192</v>
+        <v>0.2329266369342804</v>
       </c>
       <c r="DP5" t="n">
         <v>0.2270579189062119</v>
@@ -3968,7 +3970,7 @@
         <v>0.2195329219102859</v>
       </c>
       <c r="DS5" t="n">
-        <v>0.2165657877922058</v>
+        <v>0.2165658175945282</v>
       </c>
       <c r="DT5" t="n">
         <v>0.2118554562330246</v>
@@ -3977,22 +3979,22 @@
         <v>0.2103708535432816</v>
       </c>
       <c r="DV5" t="n">
-        <v>0.2127471417188644</v>
+        <v>0.2127471566200256</v>
       </c>
       <c r="DW5" t="n">
         <v>0.2148200124502182</v>
       </c>
       <c r="DX5" t="n">
-        <v>0.2688837349414825</v>
+        <v>0.2688837647438049</v>
       </c>
       <c r="DY5" t="n">
-        <v>0.2588129937648773</v>
+        <v>0.2588130235671997</v>
       </c>
       <c r="DZ5" t="n">
         <v>0.2573569416999817</v>
       </c>
       <c r="EA5" t="n">
-        <v>0.2498797178268433</v>
+        <v>0.2498797327280045</v>
       </c>
       <c r="EB5" t="n">
         <v>0.2491326779127121</v>
@@ -4007,7 +4009,7 @@
         <v>0.238980308175087</v>
       </c>
       <c r="EF5" t="n">
-        <v>0.236628070473671</v>
+        <v>0.2366280853748322</v>
       </c>
       <c r="EG5" t="n">
         <v>0.2345291972160339</v>
@@ -4076,7 +4078,7 @@
         <v>0.2749622166156769</v>
       </c>
       <c r="FC5" t="n">
-        <v>0.2773380875587463</v>
+        <v>0.2773381173610687</v>
       </c>
       <c r="FD5" t="n">
         <v>0.2677676975727081</v>
@@ -4100,7 +4102,7 @@
         <v>0.2621167302131653</v>
       </c>
       <c r="FK5" t="n">
-        <v>0.2640602290630341</v>
+        <v>0.2640602588653564</v>
       </c>
       <c r="FL5" t="n">
         <v>0.2738323211669922</v>
@@ -4109,7 +4111,7 @@
         <v>0.2841176986694336</v>
       </c>
       <c r="FN5" t="n">
-        <v>0.2892331480979919</v>
+        <v>0.2892331779003143</v>
       </c>
       <c r="FO5" t="n">
         <v>0.289486825466156</v>
@@ -4118,7 +4120,7 @@
         <v>0.2814616560935974</v>
       </c>
       <c r="FQ5" t="n">
-        <v>0.2795988917350769</v>
+        <v>0.2795989215373993</v>
       </c>
       <c r="FR5" t="n">
         <v>0.2849221229553223</v>
@@ -4127,7 +4129,7 @@
         <v>0.2826381623744965</v>
       </c>
       <c r="FT5" t="n">
-        <v>0.2828284204006195</v>
+        <v>0.2828284502029419</v>
       </c>
       <c r="FU5" t="n">
         <v>0.2808769345283508</v>
@@ -4169,7 +4171,7 @@
         <v>0.3037469387054443</v>
       </c>
       <c r="GH5" t="n">
-        <v>0.3000350296497345</v>
+        <v>0.3000350594520569</v>
       </c>
       <c r="GI5" t="n">
         <v>0.3007134795188904</v>
@@ -4193,7 +4195,7 @@
         <v>0.3410508632659912</v>
       </c>
       <c r="GP5" t="n">
-        <v>0.3339481055736542</v>
+        <v>0.3339481353759766</v>
       </c>
       <c r="GQ5" t="n">
         <v>0.3309441804885864</v>
@@ -4205,7 +4207,7 @@
         <v>0.3282979726791382</v>
       </c>
       <c r="GT5" t="n">
-        <v>0.3296602666378021</v>
+        <v>0.3296602964401245</v>
       </c>
       <c r="GU5" t="n">
         <v>0.3239479064941406</v>
@@ -4217,31 +4219,31 @@
         <v>0.3242652416229248</v>
       </c>
       <c r="GX5" t="n">
-        <v>0.3253836929798126</v>
+        <v>0.325383722782135</v>
       </c>
       <c r="GY5" t="n">
-        <v>0.3256891667842865</v>
+        <v>0.3256891965866089</v>
       </c>
       <c r="GZ5" t="n">
-        <v>0.3388771116733551</v>
+        <v>0.3388771414756775</v>
       </c>
       <c r="HA5" t="n">
         <v>0.3517445623874664</v>
       </c>
       <c r="HB5" t="n">
-        <v>0.3643373250961304</v>
+        <v>0.3643373548984528</v>
       </c>
       <c r="HC5" t="n">
-        <v>0.3583309054374695</v>
+        <v>0.3583309352397919</v>
       </c>
       <c r="HD5" t="n">
         <v>0.3469274640083313</v>
       </c>
       <c r="HE5" t="n">
-        <v>0.3420506119728088</v>
+        <v>0.3420506715774536</v>
       </c>
       <c r="HF5" t="n">
-        <v>0.3436167240142822</v>
+        <v>0.3436167538166046</v>
       </c>
       <c r="HG5" t="n">
         <v>0.3501987755298615</v>
@@ -4250,13 +4252,13 @@
         <v>0.3490679562091827</v>
       </c>
       <c r="HI5" t="n">
-        <v>0.3474437296390533</v>
+        <v>0.3474437594413757</v>
       </c>
       <c r="HJ5" t="n">
         <v>0.3500360250473022</v>
       </c>
       <c r="HK5" t="n">
-        <v>0.3437706828117371</v>
+        <v>0.3437707126140594</v>
       </c>
       <c r="HL5" t="n">
         <v>0.3455227017402649</v>
@@ -4274,10 +4276,12 @@
         <v>0.3593225479125977</v>
       </c>
       <c r="HQ5" t="n">
-        <v>0.3474158048629761</v>
-      </c>
-      <c r="HR5" s="1" t="n">
-        <v>55515</v>
+        <v>0.3474158346652985</v>
+      </c>
+      <c r="HR5" t="inlineStr">
+        <is>
+          <t>29/12/2051</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -4287,31 +4291,31 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.02522354014217854</v>
+        <v>0.02522354759275913</v>
       </c>
       <c r="C6" t="n">
-        <v>0.03395713865756989</v>
+        <v>0.03395714238286018</v>
       </c>
       <c r="D6" t="n">
-        <v>0.03604546934366226</v>
+        <v>0.03604547306895256</v>
       </c>
       <c r="E6" t="n">
-        <v>0.03757196664810181</v>
+        <v>0.0375719778239727</v>
       </c>
       <c r="F6" t="n">
-        <v>0.03801929205656052</v>
+        <v>0.03801929950714111</v>
       </c>
       <c r="G6" t="n">
-        <v>0.03728371113538742</v>
+        <v>0.03728371486067772</v>
       </c>
       <c r="H6" t="n">
-        <v>0.03668216243386269</v>
+        <v>0.03668216615915298</v>
       </c>
       <c r="I6" t="n">
-        <v>0.03632709756493568</v>
+        <v>0.03632710501551628</v>
       </c>
       <c r="J6" t="n">
-        <v>0.03652737662196159</v>
+        <v>0.03652738034725189</v>
       </c>
       <c r="K6" t="n">
         <v>0.03582604974508286</v>
@@ -4320,7 +4324,7 @@
         <v>0.03475445881485939</v>
       </c>
       <c r="M6" t="n">
-        <v>0.03368915989995003</v>
+        <v>0.03368916362524033</v>
       </c>
       <c r="N6" t="n">
         <v>0.033602524548769</v>
@@ -4329,28 +4333,28 @@
         <v>0.03417399153113365</v>
       </c>
       <c r="P6" t="n">
-        <v>0.05067431181669235</v>
+        <v>0.05067432299256325</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.06207230687141418</v>
+        <v>0.06207231432199478</v>
       </c>
       <c r="R6" t="n">
-        <v>0.06484448164701462</v>
+        <v>0.06484449654817581</v>
       </c>
       <c r="S6" t="n">
         <v>0.06573161482810974</v>
       </c>
       <c r="T6" t="n">
-        <v>0.06695108860731125</v>
+        <v>0.06695109605789185</v>
       </c>
       <c r="U6" t="n">
-        <v>0.06452777981758118</v>
+        <v>0.06452778726816177</v>
       </c>
       <c r="V6" t="n">
-        <v>0.06533069163560867</v>
+        <v>0.06533069908618927</v>
       </c>
       <c r="W6" t="n">
-        <v>0.06482532620429993</v>
+        <v>0.06482533365488052</v>
       </c>
       <c r="X6" t="n">
         <v>0.06428014487028122</v>
@@ -4359,112 +4363,112 @@
         <v>0.06382252275943756</v>
       </c>
       <c r="Z6" t="n">
-        <v>0.06065203621983528</v>
+        <v>0.06065203994512558</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.05830798670649529</v>
+        <v>0.05830799415707588</v>
       </c>
       <c r="AB6" t="n">
-        <v>0.05814253911375999</v>
+        <v>0.05814255028963089</v>
       </c>
       <c r="AC6" t="n">
-        <v>0.05953730270266533</v>
+        <v>0.05953731015324593</v>
       </c>
       <c r="AD6" t="n">
-        <v>0.08252640813589096</v>
+        <v>0.08252641558647156</v>
       </c>
       <c r="AE6" t="n">
-        <v>0.09453823417425156</v>
+        <v>0.09453824162483215</v>
       </c>
       <c r="AF6" t="n">
-        <v>0.09459768235683441</v>
+        <v>0.0945977047085762</v>
       </c>
       <c r="AG6" t="n">
-        <v>0.09646134078502655</v>
+        <v>0.09646135568618774</v>
       </c>
       <c r="AH6" t="n">
-        <v>0.09666330367326736</v>
+        <v>0.09666331112384796</v>
       </c>
       <c r="AI6" t="n">
-        <v>0.09592657536268234</v>
+        <v>0.09592658281326294</v>
       </c>
       <c r="AJ6" t="n">
-        <v>0.09270170331001282</v>
+        <v>0.09270171076059341</v>
       </c>
       <c r="AK6" t="n">
-        <v>0.09166421741247177</v>
+        <v>0.09166423231363297</v>
       </c>
       <c r="AL6" t="n">
-        <v>0.09194351732730865</v>
+        <v>0.09194352477788925</v>
       </c>
       <c r="AM6" t="n">
-        <v>0.0888768658041954</v>
+        <v>0.088876873254776</v>
       </c>
       <c r="AN6" t="n">
-        <v>0.08451274782419205</v>
+        <v>0.08451275527477264</v>
       </c>
       <c r="AO6" t="n">
-        <v>0.08248945325613022</v>
+        <v>0.08248946070671082</v>
       </c>
       <c r="AP6" t="n">
         <v>0.08469582349061966</v>
       </c>
       <c r="AQ6" t="n">
-        <v>0.08537336438894272</v>
+        <v>0.08537337183952332</v>
       </c>
       <c r="AR6" t="n">
-        <v>0.1118640378117561</v>
+        <v>0.1118640527129173</v>
       </c>
       <c r="AS6" t="n">
-        <v>0.1191564276814461</v>
+        <v>0.1191564351320267</v>
       </c>
       <c r="AT6" t="n">
-        <v>0.1197955384850502</v>
+        <v>0.1197955459356308</v>
       </c>
       <c r="AU6" t="n">
-        <v>0.1211981922388077</v>
+        <v>0.1211981996893883</v>
       </c>
       <c r="AV6" t="n">
-        <v>0.1193279400467873</v>
+        <v>0.1193279549479485</v>
       </c>
       <c r="AW6" t="n">
-        <v>0.1149034574627876</v>
+        <v>0.1149034649133682</v>
       </c>
       <c r="AX6" t="n">
-        <v>0.1153632625937462</v>
+        <v>0.1153632700443268</v>
       </c>
       <c r="AY6" t="n">
-        <v>0.1144291609525681</v>
+        <v>0.1144291684031487</v>
       </c>
       <c r="AZ6" t="n">
-        <v>0.1130299717187881</v>
+        <v>0.1130299791693687</v>
       </c>
       <c r="BA6" t="n">
-        <v>0.1092603504657745</v>
+        <v>0.1092603579163551</v>
       </c>
       <c r="BB6" t="n">
-        <v>0.1044370457530022</v>
+        <v>0.1044370532035828</v>
       </c>
       <c r="BC6" t="n">
-        <v>0.1027124673128128</v>
+        <v>0.1027124747633934</v>
       </c>
       <c r="BD6" t="n">
         <v>0.10142582654953</v>
       </c>
       <c r="BE6" t="n">
-        <v>0.1044525802135468</v>
+        <v>0.1044525876641273</v>
       </c>
       <c r="BF6" t="n">
-        <v>0.1403848528862</v>
+        <v>0.1403848677873611</v>
       </c>
       <c r="BG6" t="n">
-        <v>0.1427127420902252</v>
+        <v>0.1427127718925476</v>
       </c>
       <c r="BH6" t="n">
         <v>0.142006054520607</v>
       </c>
       <c r="BI6" t="n">
-        <v>0.1385051906108856</v>
+        <v>0.1385052055120468</v>
       </c>
       <c r="BJ6" t="n">
         <v>0.1386381387710571</v>
@@ -4476,37 +4480,37 @@
         <v>0.1316160708665848</v>
       </c>
       <c r="BM6" t="n">
-        <v>0.1290475577116013</v>
+        <v>0.1290475726127625</v>
       </c>
       <c r="BN6" t="n">
-        <v>0.1271607130765915</v>
+        <v>0.1271607279777527</v>
       </c>
       <c r="BO6" t="n">
         <v>0.1283615678548813</v>
       </c>
       <c r="BP6" t="n">
-        <v>0.120036356151104</v>
+        <v>0.1200363636016846</v>
       </c>
       <c r="BQ6" t="n">
-        <v>0.1193666011095047</v>
+        <v>0.1193666085600853</v>
       </c>
       <c r="BR6" t="n">
         <v>0.1187366172671318</v>
       </c>
       <c r="BS6" t="n">
-        <v>0.1185799688100815</v>
+        <v>0.1185799762606621</v>
       </c>
       <c r="BT6" t="n">
-        <v>0.1758566647768021</v>
+        <v>0.1758566796779633</v>
       </c>
       <c r="BU6" t="n">
-        <v>0.1738847196102142</v>
+        <v>0.1738847345113754</v>
       </c>
       <c r="BV6" t="n">
-        <v>0.1697055399417877</v>
+        <v>0.1697055548429489</v>
       </c>
       <c r="BW6" t="n">
-        <v>0.169389545917511</v>
+        <v>0.1693895608186722</v>
       </c>
       <c r="BX6" t="n">
         <v>0.1673218011856079</v>
@@ -4533,31 +4537,31 @@
         <v>0.1392474919557571</v>
       </c>
       <c r="CF6" t="n">
-        <v>0.139367938041687</v>
+        <v>0.1393679529428482</v>
       </c>
       <c r="CG6" t="n">
         <v>0.1426165997982025</v>
       </c>
       <c r="CH6" t="n">
-        <v>0.2018893212080002</v>
+        <v>0.2018893510103226</v>
       </c>
       <c r="CI6" t="n">
-        <v>0.1999574303627014</v>
+        <v>0.1999574452638626</v>
       </c>
       <c r="CJ6" t="n">
-        <v>0.1969169080257416</v>
+        <v>0.196916937828064</v>
       </c>
       <c r="CK6" t="n">
-        <v>0.1926058828830719</v>
+        <v>0.1926058977842331</v>
       </c>
       <c r="CL6" t="n">
-        <v>0.1889018565416336</v>
+        <v>0.1889018714427948</v>
       </c>
       <c r="CM6" t="n">
-        <v>0.1820531785488129</v>
+        <v>0.1820531934499741</v>
       </c>
       <c r="CN6" t="n">
-        <v>0.1825180053710938</v>
+        <v>0.1825180202722549</v>
       </c>
       <c r="CO6" t="n">
         <v>0.1760341227054596</v>
@@ -4566,13 +4570,13 @@
         <v>0.1743953078985214</v>
       </c>
       <c r="CQ6" t="n">
-        <v>0.1750194877386093</v>
+        <v>0.1750195026397705</v>
       </c>
       <c r="CR6" t="n">
-        <v>0.1620153784751892</v>
+        <v>0.1620153933763504</v>
       </c>
       <c r="CS6" t="n">
-        <v>0.1594205647706985</v>
+        <v>0.1594205796718597</v>
       </c>
       <c r="CT6" t="n">
         <v>0.1593927592039108</v>
@@ -4581,34 +4585,34 @@
         <v>0.1656244844198227</v>
       </c>
       <c r="CV6" t="n">
-        <v>0.2375306189060211</v>
+        <v>0.2375306338071823</v>
       </c>
       <c r="CW6" t="n">
-        <v>0.225055143237114</v>
+        <v>0.2250551581382751</v>
       </c>
       <c r="CX6" t="n">
-        <v>0.2246175706386566</v>
+        <v>0.2246175855398178</v>
       </c>
       <c r="CY6" t="n">
         <v>0.2229142487049103</v>
       </c>
       <c r="CZ6" t="n">
-        <v>0.2134500592947006</v>
+        <v>0.2134500741958618</v>
       </c>
       <c r="DA6" t="n">
-        <v>0.209853321313858</v>
+        <v>0.2098533362150192</v>
       </c>
       <c r="DB6" t="n">
-        <v>0.2101660370826721</v>
+        <v>0.2101660519838333</v>
       </c>
       <c r="DC6" t="n">
         <v>0.2054412215948105</v>
       </c>
       <c r="DD6" t="n">
-        <v>0.2048725783824921</v>
+        <v>0.2048725932836533</v>
       </c>
       <c r="DE6" t="n">
-        <v>0.1992050260305405</v>
+        <v>0.1992050409317017</v>
       </c>
       <c r="DF6" t="n">
         <v>0.19318488240242</v>
@@ -4632,13 +4636,13 @@
         <v>0.2422073781490326</v>
       </c>
       <c r="DM6" t="n">
-        <v>0.240484282374382</v>
+        <v>0.2404842972755432</v>
       </c>
       <c r="DN6" t="n">
-        <v>0.2333645075559616</v>
+        <v>0.2333645224571228</v>
       </c>
       <c r="DO6" t="n">
-        <v>0.23412124812603</v>
+        <v>0.2341212630271912</v>
       </c>
       <c r="DP6" t="n">
         <v>0.2281384170055389</v>
@@ -4662,10 +4666,10 @@
         <v>0.2134488672018051</v>
       </c>
       <c r="DW6" t="n">
-        <v>0.2155052125453949</v>
+        <v>0.2155052274465561</v>
       </c>
       <c r="DX6" t="n">
-        <v>0.2705222070217133</v>
+        <v>0.2705222368240356</v>
       </c>
       <c r="DY6" t="n">
         <v>0.2603305876255035</v>
@@ -4677,16 +4681,16 @@
         <v>0.2511501014232635</v>
       </c>
       <c r="EB6" t="n">
-        <v>0.2502939701080322</v>
+        <v>0.2502939999103546</v>
       </c>
       <c r="EC6" t="n">
-        <v>0.2443028390407562</v>
+        <v>0.2443028688430786</v>
       </c>
       <c r="ED6" t="n">
         <v>0.24149489402771</v>
       </c>
       <c r="EE6" t="n">
-        <v>0.239924356341362</v>
+        <v>0.2399243861436844</v>
       </c>
       <c r="EF6" t="n">
         <v>0.2375199049711227</v>
@@ -4713,10 +4717,10 @@
         <v>0.2767636775970459</v>
       </c>
       <c r="EN6" t="n">
-        <v>0.2724239528179169</v>
+        <v>0.2724239826202393</v>
       </c>
       <c r="EO6" t="n">
-        <v>0.2654723525047302</v>
+        <v>0.2654723823070526</v>
       </c>
       <c r="EP6" t="n">
         <v>0.268595963716507</v>
@@ -4725,7 +4729,7 @@
         <v>0.2575906217098236</v>
       </c>
       <c r="ER6" t="n">
-        <v>0.2573244273662567</v>
+        <v>0.2573244571685791</v>
       </c>
       <c r="ES6" t="n">
         <v>0.2511412501335144</v>
@@ -4734,7 +4738,7 @@
         <v>0.2539514601230621</v>
       </c>
       <c r="EU6" t="n">
-        <v>0.2530920505523682</v>
+        <v>0.2530920803546906</v>
       </c>
       <c r="EV6" t="n">
         <v>0.2495596557855606</v>
@@ -4746,7 +4750,7 @@
         <v>0.2491025924682617</v>
       </c>
       <c r="EY6" t="n">
-        <v>0.2607878744602203</v>
+        <v>0.2607879042625427</v>
       </c>
       <c r="EZ6" t="n">
         <v>0.2858297526836395</v>
@@ -4770,7 +4774,7 @@
         <v>0.2695747017860413</v>
       </c>
       <c r="FG6" t="n">
-        <v>0.2662915587425232</v>
+        <v>0.2662915885448456</v>
       </c>
       <c r="FH6" t="n">
         <v>0.2617667615413666</v>
@@ -4785,7 +4789,7 @@
         <v>0.2645911872386932</v>
       </c>
       <c r="FL6" t="n">
-        <v>0.274368554353714</v>
+        <v>0.2743685841560364</v>
       </c>
       <c r="FM6" t="n">
         <v>0.2846744060516357</v>
@@ -4797,22 +4801,22 @@
         <v>0.2901950776576996</v>
       </c>
       <c r="FP6" t="n">
-        <v>0.2821386456489563</v>
+        <v>0.2821386754512787</v>
       </c>
       <c r="FQ6" t="n">
-        <v>0.2802689075469971</v>
+        <v>0.2802689373493195</v>
       </c>
       <c r="FR6" t="n">
         <v>0.2856284379959106</v>
       </c>
       <c r="FS6" t="n">
-        <v>0.2833361029624939</v>
+        <v>0.2833361327648163</v>
       </c>
       <c r="FT6" t="n">
         <v>0.2835452556610107</v>
       </c>
       <c r="FU6" t="n">
-        <v>0.2815987169742584</v>
+        <v>0.2815987467765808</v>
       </c>
       <c r="FV6" t="n">
         <v>0.2834430634975433</v>
@@ -4827,10 +4831,10 @@
         <v>0.293546050786972</v>
       </c>
       <c r="FZ6" t="n">
-        <v>0.2979891896247864</v>
+        <v>0.2979892194271088</v>
       </c>
       <c r="GA6" t="n">
-        <v>0.3126568794250488</v>
+        <v>0.3126569092273712</v>
       </c>
       <c r="GB6" t="n">
         <v>0.3064280450344086</v>
@@ -4839,16 +4843,16 @@
         <v>0.3071700930595398</v>
       </c>
       <c r="GD6" t="n">
-        <v>0.3083421885967255</v>
+        <v>0.3083422183990479</v>
       </c>
       <c r="GE6" t="n">
-        <v>0.3083177506923676</v>
+        <v>0.3083177804946899</v>
       </c>
       <c r="GF6" t="n">
-        <v>0.3063856065273285</v>
+        <v>0.3063856363296509</v>
       </c>
       <c r="GG6" t="n">
-        <v>0.3047313094139099</v>
+        <v>0.3047313392162323</v>
       </c>
       <c r="GH6" t="n">
         <v>0.3010034561157227</v>
@@ -4857,25 +4861,25 @@
         <v>0.3016247153282166</v>
       </c>
       <c r="GJ6" t="n">
-        <v>0.3020752370357513</v>
+        <v>0.3020752668380737</v>
       </c>
       <c r="GK6" t="n">
         <v>0.3059440553188324</v>
       </c>
       <c r="GL6" t="n">
-        <v>0.312444269657135</v>
+        <v>0.3124442994594574</v>
       </c>
       <c r="GM6" t="n">
-        <v>0.3187808394432068</v>
+        <v>0.3187808692455292</v>
       </c>
       <c r="GN6" t="n">
-        <v>0.3341204524040222</v>
+        <v>0.3341204822063446</v>
       </c>
       <c r="GO6" t="n">
         <v>0.3420371115207672</v>
       </c>
       <c r="GP6" t="n">
-        <v>0.3349483609199524</v>
+        <v>0.3349483907222748</v>
       </c>
       <c r="GQ6" t="n">
         <v>0.3318676352500916</v>
@@ -4884,13 +4888,13 @@
         <v>0.3308370113372803</v>
       </c>
       <c r="GS6" t="n">
-        <v>0.3292349576950073</v>
+        <v>0.3292349874973297</v>
       </c>
       <c r="GT6" t="n">
-        <v>0.3306314945220947</v>
+        <v>0.3306315243244171</v>
       </c>
       <c r="GU6" t="n">
-        <v>0.3249135613441467</v>
+        <v>0.3249135911464691</v>
       </c>
       <c r="GV6" t="n">
         <v>0.3301834464073181</v>
@@ -4902,7 +4906,7 @@
         <v>0.3264118134975433</v>
       </c>
       <c r="GY6" t="n">
-        <v>0.3267403841018677</v>
+        <v>0.3267404139041901</v>
       </c>
       <c r="GZ6" t="n">
         <v>0.3399000763893127</v>
@@ -4911,22 +4915,22 @@
         <v>0.3527229428291321</v>
       </c>
       <c r="HB6" t="n">
-        <v>0.3654146790504456</v>
+        <v>0.3654147088527679</v>
       </c>
       <c r="HC6" t="n">
-        <v>0.3591762483119965</v>
+        <v>0.3591762781143188</v>
       </c>
       <c r="HD6" t="n">
         <v>0.3481805026531219</v>
       </c>
       <c r="HE6" t="n">
-        <v>0.3432444632053375</v>
+        <v>0.3432445228099823</v>
       </c>
       <c r="HF6" t="n">
         <v>0.3448282480239868</v>
       </c>
       <c r="HG6" t="n">
-        <v>0.3514571487903595</v>
+        <v>0.3514571785926819</v>
       </c>
       <c r="HH6" t="n">
         <v>0.3503752946853638</v>
@@ -4935,31 +4939,33 @@
         <v>0.3487776517868042</v>
       </c>
       <c r="HJ6" t="n">
-        <v>0.3514176309108734</v>
+        <v>0.3514176607131958</v>
       </c>
       <c r="HK6" t="n">
-        <v>0.3451667428016663</v>
+        <v>0.345166802406311</v>
       </c>
       <c r="HL6" t="n">
         <v>0.3469631969928741</v>
       </c>
       <c r="HM6" t="n">
-        <v>0.3439945876598358</v>
+        <v>0.3439946472644806</v>
       </c>
       <c r="HN6" t="n">
         <v>0.3671712577342987</v>
       </c>
       <c r="HO6" t="n">
-        <v>0.3814215958118439</v>
+        <v>0.3814216256141663</v>
       </c>
       <c r="HP6" t="n">
-        <v>0.3603777885437012</v>
+        <v>0.3603778183460236</v>
       </c>
       <c r="HQ6" t="n">
         <v>0.3481786847114563</v>
       </c>
-      <c r="HR6" s="1" t="n">
-        <v>55516</v>
+      <c r="HR6" t="inlineStr">
+        <is>
+          <t>30/12/2051</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -4969,10 +4975,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.02562805451452732</v>
+        <v>0.02562805823981762</v>
       </c>
       <c r="C7" t="n">
-        <v>0.03436929360032082</v>
+        <v>0.03436929732561111</v>
       </c>
       <c r="D7" t="n">
         <v>0.03644922748208046</v>
@@ -4981,37 +4987,37 @@
         <v>0.03796205297112465</v>
       </c>
       <c r="F7" t="n">
-        <v>0.03838392347097397</v>
+        <v>0.03838392719626427</v>
       </c>
       <c r="G7" t="n">
-        <v>0.03762638941407204</v>
+        <v>0.03762639313936234</v>
       </c>
       <c r="H7" t="n">
-        <v>0.03700553998351097</v>
+        <v>0.03700554370880127</v>
       </c>
       <c r="I7" t="n">
         <v>0.03664589673280716</v>
       </c>
       <c r="J7" t="n">
-        <v>0.03683914616703987</v>
+        <v>0.03683914989233017</v>
       </c>
       <c r="K7" t="n">
-        <v>0.03612423315644264</v>
+        <v>0.03612423688173294</v>
       </c>
       <c r="L7" t="n">
-        <v>0.03502486273646355</v>
+        <v>0.03502486646175385</v>
       </c>
       <c r="M7" t="n">
-        <v>0.03393165394663811</v>
+        <v>0.03393165767192841</v>
       </c>
       <c r="N7" t="n">
         <v>0.03384201601147652</v>
       </c>
       <c r="O7" t="n">
-        <v>0.03441000357270241</v>
+        <v>0.03441000729799271</v>
       </c>
       <c r="P7" t="n">
-        <v>0.0513003021478653</v>
+        <v>0.05130030587315559</v>
       </c>
       <c r="Q7" t="n">
         <v>0.06270501762628555</v>
@@ -5020,10 +5026,10 @@
         <v>0.06548599153757095</v>
       </c>
       <c r="S7" t="n">
-        <v>0.06631483137607574</v>
+        <v>0.06631483882665634</v>
       </c>
       <c r="T7" t="n">
-        <v>0.06752477586269379</v>
+        <v>0.06752478331327438</v>
       </c>
       <c r="U7" t="n">
         <v>0.06504668295383453</v>
@@ -5038,19 +5044,19 @@
         <v>0.06474866718053818</v>
       </c>
       <c r="Y7" t="n">
-        <v>0.06426893174648285</v>
+        <v>0.06426893919706345</v>
       </c>
       <c r="Z7" t="n">
-        <v>0.06105054169893265</v>
+        <v>0.06105054542422295</v>
       </c>
       <c r="AA7" t="n">
-        <v>0.05867773294448853</v>
+        <v>0.05867774039506912</v>
       </c>
       <c r="AB7" t="n">
-        <v>0.0585140734910965</v>
+        <v>0.05851408094167709</v>
       </c>
       <c r="AC7" t="n">
-        <v>0.05990136787295341</v>
+        <v>0.05990137532353401</v>
       </c>
       <c r="AD7" t="n">
         <v>0.08329813182353973</v>
@@ -5062,58 +5068,58 @@
         <v>0.09540054947137833</v>
       </c>
       <c r="AG7" t="n">
-        <v>0.09717480093240738</v>
+        <v>0.09717480838298798</v>
       </c>
       <c r="AH7" t="n">
-        <v>0.09735792875289917</v>
+        <v>0.09735793620347977</v>
       </c>
       <c r="AI7" t="n">
-        <v>0.09658827632665634</v>
+        <v>0.09658828377723694</v>
       </c>
       <c r="AJ7" t="n">
         <v>0.09331237524747849</v>
       </c>
       <c r="AK7" t="n">
-        <v>0.09223896265029907</v>
+        <v>0.09223897010087967</v>
       </c>
       <c r="AL7" t="n">
         <v>0.09251928329467773</v>
       </c>
       <c r="AM7" t="n">
-        <v>0.08941950649023056</v>
+        <v>0.08941951394081116</v>
       </c>
       <c r="AN7" t="n">
         <v>0.08498422801494598</v>
       </c>
       <c r="AO7" t="n">
-        <v>0.08293697237968445</v>
+        <v>0.08293697983026505</v>
       </c>
       <c r="AP7" t="n">
         <v>0.08515981584787369</v>
       </c>
       <c r="AQ7" t="n">
-        <v>0.08582130074501038</v>
+        <v>0.08582130819559097</v>
       </c>
       <c r="AR7" t="n">
         <v>0.1127525791525841</v>
       </c>
       <c r="AS7" t="n">
-        <v>0.1201004907488823</v>
+        <v>0.1201004981994629</v>
       </c>
       <c r="AT7" t="n">
-        <v>0.1206775680184364</v>
+        <v>0.120677575469017</v>
       </c>
       <c r="AU7" t="n">
-        <v>0.1219590157270432</v>
+        <v>0.1219590306282043</v>
       </c>
       <c r="AV7" t="n">
-        <v>0.1201567947864532</v>
+        <v>0.1201568022370338</v>
       </c>
       <c r="AW7" t="n">
-        <v>0.1156130060553551</v>
+        <v>0.1156130135059357</v>
       </c>
       <c r="AX7" t="n">
-        <v>0.1160600632429123</v>
+        <v>0.1160600781440735</v>
       </c>
       <c r="AY7" t="n">
         <v>0.1150865480303764</v>
@@ -5122,19 +5128,19 @@
         <v>0.1136777251958847</v>
       </c>
       <c r="BA7" t="n">
-        <v>0.1098615154623985</v>
+        <v>0.1098615229129791</v>
       </c>
       <c r="BB7" t="n">
-        <v>0.1049540415406227</v>
+        <v>0.1049540489912033</v>
       </c>
       <c r="BC7" t="n">
         <v>0.103217288851738</v>
       </c>
       <c r="BD7" t="n">
-        <v>0.1019349172711372</v>
+        <v>0.1019349247217178</v>
       </c>
       <c r="BE7" t="n">
-        <v>0.1049547269940376</v>
+        <v>0.1049547344446182</v>
       </c>
       <c r="BF7" t="n">
         <v>0.1413466781377792</v>
@@ -5146,13 +5152,13 @@
         <v>0.1429286599159241</v>
       </c>
       <c r="BI7" t="n">
-        <v>0.1393507570028305</v>
+        <v>0.1393507719039917</v>
       </c>
       <c r="BJ7" t="n">
         <v>0.1395094394683838</v>
       </c>
       <c r="BK7" t="n">
-        <v>0.1330464035272598</v>
+        <v>0.133046418428421</v>
       </c>
       <c r="BL7" t="n">
         <v>0.1323313266038895</v>
@@ -5164,19 +5170,19 @@
         <v>0.1278405636548996</v>
       </c>
       <c r="BO7" t="n">
-        <v>0.1290033757686615</v>
+        <v>0.1290033906698227</v>
       </c>
       <c r="BP7" t="n">
-        <v>0.1205901727080345</v>
+        <v>0.1205901801586151</v>
       </c>
       <c r="BQ7" t="n">
-        <v>0.119907982647419</v>
+        <v>0.1199079975485802</v>
       </c>
       <c r="BR7" t="n">
-        <v>0.1192829310894012</v>
+        <v>0.1192829385399818</v>
       </c>
       <c r="BS7" t="n">
-        <v>0.1191109493374825</v>
+        <v>0.119110956788063</v>
       </c>
       <c r="BT7" t="n">
         <v>0.1771750897169113</v>
@@ -5185,31 +5191,31 @@
         <v>0.1751107722520828</v>
       </c>
       <c r="BV7" t="n">
-        <v>0.1709050685167313</v>
+        <v>0.1709050834178925</v>
       </c>
       <c r="BW7" t="n">
-        <v>0.1704538315534592</v>
+        <v>0.1704538464546204</v>
       </c>
       <c r="BX7" t="n">
-        <v>0.1682902723550797</v>
+        <v>0.1682902872562408</v>
       </c>
       <c r="BY7" t="n">
         <v>0.164189800620079</v>
       </c>
       <c r="BZ7" t="n">
-        <v>0.1600387543439865</v>
+        <v>0.1600387692451477</v>
       </c>
       <c r="CA7" t="n">
-        <v>0.1570315659046173</v>
+        <v>0.1570315808057785</v>
       </c>
       <c r="CB7" t="n">
-        <v>0.1548685133457184</v>
+        <v>0.1548685282468796</v>
       </c>
       <c r="CC7" t="n">
-        <v>0.1505695879459381</v>
+        <v>0.1505696028470993</v>
       </c>
       <c r="CD7" t="n">
-        <v>0.1466484367847443</v>
+        <v>0.1466484516859055</v>
       </c>
       <c r="CE7" t="n">
         <v>0.1398404389619827</v>
@@ -5218,40 +5224,40 @@
         <v>0.1399616748094559</v>
       </c>
       <c r="CG7" t="n">
-        <v>0.143212616443634</v>
+        <v>0.1432126313447952</v>
       </c>
       <c r="CH7" t="n">
-        <v>0.2032133936882019</v>
+        <v>0.2032134085893631</v>
       </c>
       <c r="CI7" t="n">
-        <v>0.2013147175312042</v>
+        <v>0.2013147324323654</v>
       </c>
       <c r="CJ7" t="n">
-        <v>0.1981805264949799</v>
+        <v>0.1981805562973022</v>
       </c>
       <c r="CK7" t="n">
         <v>0.1937174201011658</v>
       </c>
       <c r="CL7" t="n">
-        <v>0.1899826973676682</v>
+        <v>0.1899827122688293</v>
       </c>
       <c r="CM7" t="n">
-        <v>0.183054506778717</v>
+        <v>0.1830545216798782</v>
       </c>
       <c r="CN7" t="n">
-        <v>0.183454766869545</v>
+        <v>0.1834547817707062</v>
       </c>
       <c r="CO7" t="n">
         <v>0.1769076287746429</v>
       </c>
       <c r="CP7" t="n">
-        <v>0.1752196848392487</v>
+        <v>0.1752196997404099</v>
       </c>
       <c r="CQ7" t="n">
-        <v>0.1757816821336746</v>
+        <v>0.1757816970348358</v>
       </c>
       <c r="CR7" t="n">
-        <v>0.1626796722412109</v>
+        <v>0.1626796871423721</v>
       </c>
       <c r="CS7" t="n">
         <v>0.1600495278835297</v>
@@ -5260,16 +5266,16 @@
         <v>0.1600085198879242</v>
       </c>
       <c r="CU7" t="n">
-        <v>0.1662711948156357</v>
+        <v>0.1662712097167969</v>
       </c>
       <c r="CV7" t="n">
-        <v>0.2388625741004944</v>
+        <v>0.2388625890016556</v>
       </c>
       <c r="CW7" t="n">
-        <v>0.2264378815889359</v>
+        <v>0.2264379113912582</v>
       </c>
       <c r="CX7" t="n">
-        <v>0.2258539795875549</v>
+        <v>0.2258539944887161</v>
       </c>
       <c r="CY7" t="n">
         <v>0.2241293787956238</v>
@@ -5281,19 +5287,19 @@
         <v>0.210890606045723</v>
       </c>
       <c r="DB7" t="n">
-        <v>0.2111420929431915</v>
+        <v>0.2111421078443527</v>
       </c>
       <c r="DC7" t="n">
         <v>0.2063076049089432</v>
       </c>
       <c r="DD7" t="n">
-        <v>0.2057186663150787</v>
+        <v>0.2057186812162399</v>
       </c>
       <c r="DE7" t="n">
         <v>0.1999949216842651</v>
       </c>
       <c r="DF7" t="n">
-        <v>0.1938789486885071</v>
+        <v>0.1938789635896683</v>
       </c>
       <c r="DG7" t="n">
         <v>0.19071364402771</v>
@@ -5302,31 +5308,31 @@
         <v>0.1894662082195282</v>
       </c>
       <c r="DI7" t="n">
-        <v>0.1920864433050156</v>
+        <v>0.1920864582061768</v>
       </c>
       <c r="DJ7" t="n">
-        <v>0.2556321024894714</v>
+        <v>0.2556321322917938</v>
       </c>
       <c r="DK7" t="n">
-        <v>0.2519600093364716</v>
+        <v>0.2519600391387939</v>
       </c>
       <c r="DL7" t="n">
         <v>0.2434325069189072</v>
       </c>
       <c r="DM7" t="n">
-        <v>0.2416587322950363</v>
+        <v>0.2416587471961975</v>
       </c>
       <c r="DN7" t="n">
-        <v>0.2344612777233124</v>
+        <v>0.2344612926244736</v>
       </c>
       <c r="DO7" t="n">
-        <v>0.2350915521383286</v>
+        <v>0.2350915670394897</v>
       </c>
       <c r="DP7" t="n">
-        <v>0.2290369272232056</v>
+        <v>0.2290369421243668</v>
       </c>
       <c r="DQ7" t="n">
-        <v>0.2229118645191193</v>
+        <v>0.2229118943214417</v>
       </c>
       <c r="DR7" t="n">
         <v>0.2212967574596405</v>
@@ -5338,22 +5344,22 @@
         <v>0.2133280038833618</v>
       </c>
       <c r="DU7" t="n">
-        <v>0.2116210907697678</v>
+        <v>0.2116211205720901</v>
       </c>
       <c r="DV7" t="n">
-        <v>0.2140780091285706</v>
+        <v>0.2140780240297318</v>
       </c>
       <c r="DW7" t="n">
         <v>0.2161291092634201</v>
       </c>
       <c r="DX7" t="n">
-        <v>0.2718741893768311</v>
+        <v>0.2718742191791534</v>
       </c>
       <c r="DY7" t="n">
         <v>0.2615775167942047</v>
       </c>
       <c r="DZ7" t="n">
-        <v>0.2600552141666412</v>
+        <v>0.2600552439689636</v>
       </c>
       <c r="EA7" t="n">
         <v>0.2521920204162598</v>
@@ -5362,22 +5368,22 @@
         <v>0.2512693107128143</v>
       </c>
       <c r="EC7" t="n">
-        <v>0.2452240288257599</v>
+        <v>0.2452240586280823</v>
       </c>
       <c r="ED7" t="n">
         <v>0.2423636168241501</v>
       </c>
       <c r="EE7" t="n">
-        <v>0.2407473772764206</v>
+        <v>0.240747407078743</v>
       </c>
       <c r="EF7" t="n">
         <v>0.2382859736680984</v>
       </c>
       <c r="EG7" t="n">
-        <v>0.2361034899950027</v>
+        <v>0.2361035197973251</v>
       </c>
       <c r="EH7" t="n">
-        <v>0.2240142971277237</v>
+        <v>0.2240143269300461</v>
       </c>
       <c r="EI7" t="n">
         <v>0.2274878025054932</v>
@@ -5392,7 +5398,7 @@
         <v>0.2813215851783752</v>
       </c>
       <c r="EM7" t="n">
-        <v>0.277779221534729</v>
+        <v>0.2777792513370514</v>
       </c>
       <c r="EN7" t="n">
         <v>0.273372083902359</v>
@@ -5404,46 +5410,46 @@
         <v>0.2694180011749268</v>
       </c>
       <c r="EQ7" t="n">
-        <v>0.2583473324775696</v>
+        <v>0.258347362279892</v>
       </c>
       <c r="ER7" t="n">
         <v>0.2581373155117035</v>
       </c>
       <c r="ES7" t="n">
-        <v>0.2518907785415649</v>
+        <v>0.2518908083438873</v>
       </c>
       <c r="ET7" t="n">
         <v>0.2546548247337341</v>
       </c>
       <c r="EU7" t="n">
-        <v>0.2537471652030945</v>
+        <v>0.2537471950054169</v>
       </c>
       <c r="EV7" t="n">
-        <v>0.2501920759677887</v>
+        <v>0.2501921057701111</v>
       </c>
       <c r="EW7" t="n">
         <v>0.249899834394455</v>
       </c>
       <c r="EX7" t="n">
-        <v>0.2496478110551834</v>
+        <v>0.2496478408575058</v>
       </c>
       <c r="EY7" t="n">
         <v>0.2614216208457947</v>
       </c>
       <c r="EZ7" t="n">
-        <v>0.2865191698074341</v>
+        <v>0.2865191996097565</v>
       </c>
       <c r="FA7" t="n">
-        <v>0.2870573699474335</v>
+        <v>0.2870573997497559</v>
       </c>
       <c r="FB7" t="n">
         <v>0.2763241529464722</v>
       </c>
       <c r="FC7" t="n">
-        <v>0.2786831855773926</v>
+        <v>0.278683215379715</v>
       </c>
       <c r="FD7" t="n">
-        <v>0.2690457403659821</v>
+        <v>0.2690457701683044</v>
       </c>
       <c r="FE7" t="n">
         <v>0.2705353200435638</v>
@@ -5455,46 +5461,46 @@
         <v>0.2669112980365753</v>
       </c>
       <c r="FH7" t="n">
-        <v>0.2623741030693054</v>
+        <v>0.2623741328716278</v>
       </c>
       <c r="FI7" t="n">
-        <v>0.2610801458358765</v>
+        <v>0.2610801756381989</v>
       </c>
       <c r="FJ7" t="n">
         <v>0.263323575258255</v>
       </c>
       <c r="FK7" t="n">
-        <v>0.2651333510875702</v>
+        <v>0.2651333808898926</v>
       </c>
       <c r="FL7" t="n">
-        <v>0.2749322950839996</v>
+        <v>0.274932324886322</v>
       </c>
       <c r="FM7" t="n">
         <v>0.2852621674537659</v>
       </c>
       <c r="FN7" t="n">
-        <v>0.2907228469848633</v>
+        <v>0.2907228767871857</v>
       </c>
       <c r="FO7" t="n">
         <v>0.2908971905708313</v>
       </c>
       <c r="FP7" t="n">
-        <v>0.2828101217746735</v>
+        <v>0.2828101515769958</v>
       </c>
       <c r="FQ7" t="n">
         <v>0.2809380292892456</v>
       </c>
       <c r="FR7" t="n">
-        <v>0.2863253653049469</v>
+        <v>0.2863253951072693</v>
       </c>
       <c r="FS7" t="n">
         <v>0.2840283215045929</v>
       </c>
       <c r="FT7" t="n">
-        <v>0.2842506766319275</v>
+        <v>0.2842507064342499</v>
       </c>
       <c r="FU7" t="n">
-        <v>0.2823091149330139</v>
+        <v>0.2823091447353363</v>
       </c>
       <c r="FV7" t="n">
         <v>0.2841607928276062</v>
@@ -5506,7 +5512,7 @@
         <v>0.2836199998855591</v>
       </c>
       <c r="FY7" t="n">
-        <v>0.2942115366458893</v>
+        <v>0.2942115664482117</v>
       </c>
       <c r="FZ7" t="n">
         <v>0.2987015247344971</v>
@@ -5521,37 +5527,37 @@
         <v>0.3080988228321075</v>
       </c>
       <c r="GD7" t="n">
-        <v>0.3093124032020569</v>
+        <v>0.3093124330043793</v>
       </c>
       <c r="GE7" t="n">
         <v>0.3092990219593048</v>
       </c>
       <c r="GF7" t="n">
-        <v>0.3073403835296631</v>
+        <v>0.3073404133319855</v>
       </c>
       <c r="GG7" t="n">
-        <v>0.3056668043136597</v>
+        <v>0.3056668341159821</v>
       </c>
       <c r="GH7" t="n">
-        <v>0.301918625831604</v>
+        <v>0.3019186556339264</v>
       </c>
       <c r="GI7" t="n">
-        <v>0.3025008738040924</v>
+        <v>0.3025009036064148</v>
       </c>
       <c r="GJ7" t="n">
         <v>0.3030033707618713</v>
       </c>
       <c r="GK7" t="n">
-        <v>0.306885302066803</v>
+        <v>0.3068853318691254</v>
       </c>
       <c r="GL7" t="n">
-        <v>0.3133550584316254</v>
+        <v>0.3133550882339478</v>
       </c>
       <c r="GM7" t="n">
         <v>0.3196729421615601</v>
       </c>
       <c r="GN7" t="n">
-        <v>0.3350435495376587</v>
+        <v>0.3350435793399811</v>
       </c>
       <c r="GO7" t="n">
         <v>0.3430327475070953</v>
@@ -5563,85 +5569,87 @@
         <v>0.3327821493148804</v>
       </c>
       <c r="GR7" t="n">
-        <v>0.3317412436008453</v>
+        <v>0.3317412734031677</v>
       </c>
       <c r="GS7" t="n">
-        <v>0.3301486968994141</v>
+        <v>0.3301487267017365</v>
       </c>
       <c r="GT7" t="n">
         <v>0.3315800726413727</v>
       </c>
       <c r="GU7" t="n">
-        <v>0.3258622288703918</v>
+        <v>0.3258622586727142</v>
       </c>
       <c r="GV7" t="n">
         <v>0.3311708867549896</v>
       </c>
       <c r="GW7" t="n">
-        <v>0.3262558877468109</v>
+        <v>0.3262559175491333</v>
       </c>
       <c r="GX7" t="n">
-        <v>0.3274384438991547</v>
+        <v>0.3274384737014771</v>
       </c>
       <c r="GY7" t="n">
         <v>0.3277903199195862</v>
       </c>
       <c r="GZ7" t="n">
-        <v>0.340947687625885</v>
+        <v>0.3409477174282074</v>
       </c>
       <c r="HA7" t="n">
-        <v>0.3537092208862305</v>
+        <v>0.3537092506885529</v>
       </c>
       <c r="HB7" t="n">
-        <v>0.3665052354335785</v>
+        <v>0.3665052652359009</v>
       </c>
       <c r="HC7" t="n">
         <v>0.3600437939167023</v>
       </c>
       <c r="HD7" t="n">
-        <v>0.349468857049942</v>
+        <v>0.3494688868522644</v>
       </c>
       <c r="HE7" t="n">
-        <v>0.3444927632808685</v>
+        <v>0.3444928228855133</v>
       </c>
       <c r="HF7" t="n">
-        <v>0.3460768461227417</v>
+        <v>0.3460769057273865</v>
       </c>
       <c r="HG7" t="n">
         <v>0.3527370989322662</v>
       </c>
       <c r="HH7" t="n">
-        <v>0.3516972661018372</v>
+        <v>0.3516972959041595</v>
       </c>
       <c r="HI7" t="n">
-        <v>0.3501230478286743</v>
+        <v>0.3501230776309967</v>
       </c>
       <c r="HJ7" t="n">
-        <v>0.3527966141700745</v>
+        <v>0.3527966737747192</v>
       </c>
       <c r="HK7" t="n">
-        <v>0.3465596437454224</v>
+        <v>0.3465596735477448</v>
       </c>
       <c r="HL7" t="n">
-        <v>0.3483832180500031</v>
+        <v>0.3483832478523254</v>
       </c>
       <c r="HM7" t="n">
         <v>0.3454338908195496</v>
       </c>
       <c r="HN7" t="n">
-        <v>0.3685861229896545</v>
+        <v>0.3685861527919769</v>
       </c>
       <c r="HO7" t="n">
-        <v>0.3828193247318268</v>
+        <v>0.3828193545341492</v>
       </c>
       <c r="HP7" t="n">
-        <v>0.3614596724510193</v>
+        <v>0.3614597022533417</v>
       </c>
       <c r="HQ7" t="n">
         <v>0.348989725112915</v>
       </c>
-      <c r="HR7" s="1" t="n">
-        <v>55519</v>
+      <c r="HR7" t="inlineStr">
+        <is>
+          <t>01/01/2052</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>